<commit_message>
Initial commit - Smart Task Manager
</commit_message>
<xml_diff>
--- a/exports/tasks.xlsx
+++ b/exports/tasks.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -594,7 +594,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -658,7 +658,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -690,7 +690,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>To Do</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -850,17 +850,209 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Aditi More</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>logout</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Blog Website</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Mruna Mane</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Add Task </t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Blog Website</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Mruna Mane</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Database</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Smart Planner Website</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Mruna Mane</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Implement Backend</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Smart Planner Website</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>Aditi More</t>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Mruna Mane</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>xz</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Blog Website</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0226-07-21</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Akshad Aulwar</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Dark Mode</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Blog Website</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0026-08-05</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Akshad Aulwar</t>
         </is>
       </c>
     </row>

</xml_diff>